<commit_message>
Updated prompts version, removing limits on prompts to use on Excel file. Generated outputs for just 4 files
</commit_message>
<xml_diff>
--- a/questions_v3v2_March31.xlsx
+++ b/questions_v3v2_March31.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/j_berenguer_cgiar_org/Documents/Microsoft Teams Chat Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jlbkm/document-tagging/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECC084F1-2230-4D12-9F08-3B400206A0FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D80549-890E-2D43-9EDB-064DF8B86621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2520" yWindow="1580" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Q_FOR_SCRIPT" sheetId="1" r:id="rId1"/>
@@ -36,70 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Parameter:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Year of Report.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Description:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** The date on which the study/document was published.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Output Format:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Output a single 4 digit year. E.g. "2002"</t>
-    </r>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <r>
       <t>**</t>
@@ -302,66 +239,6 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Parameter</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>:** Contributing Initiatives or centers.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Description</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">:** CGIAR is associated with multiple Initiatives and Centers. You need to extract the names of the ones mentioned in the text, if any.
-**Output Format:** Your response should be a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>string with values separated by commas</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>. For example "CIMMYT, AgriLac Resiliente, ICARDA".</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
       </rPr>
       <t>Parameter:</t>
     </r>
@@ -413,64 +290,6 @@
         <rFont val="Calibri"/>
       </rPr>
       <t>** If the CGIAR intervention focuses only on one main Impact Area, then return the name of the Impact Area (from those above), without the description in this format: "Main Area Name; No Secondary Impact Area(s)". For example: "Climate adaptation and mitigation; No Secondary Impact Area(s)". If targeting multiple Impact Areas, then your response will be the name of the applicable Impact Areas based on your internal ranking, separated by semicolors, starting from the most relevant/targeted and then going down from there. For example, if it targets two, it could be something like this: "Environmental health and biodiversity; Climate adaptation and mitigation".</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Parameter:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Country of Study.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Description:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** The name of the country where the study/observations took place.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Output Format:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Reply with the name of the country, e.g. "Spain". If the study took place in more than one country, then list the different countries separated by commas, for example "Ghana, Ethiopia"</t>
     </r>
   </si>
   <si>
@@ -587,73 +406,17 @@
 **Output Format:** Your response should be a string with values separated by commas.</t>
   </si>
   <si>
-    <r>
-      <t>**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Parameter:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Indicator measured; Unit of measure; and Result reported.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Description</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>:** Some studies use/report an Indicator to assess the impact/outcome of CGIAR interventions, as a way to measure it. Go through the content and identify the Indicator used, and then identify what unit/metric is used to measure it, and then identify its value. For example:
-- "Increase in farmable land; hectares; 3"
-The unit/metric and its associated value will be whatever is used to measure the Indicator.
-Select only the indicators and associated results that are statistically significant. There are some studies where Indicators are not reported, when this is the case you should reply with "Not reported; NA; NA"
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Output Format:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** When an Indicator is reported and identified, return the name, unit of measure, and value like this "Name; Unit of measure; Value". For example "Increase in gender engagement; Number of women; 1300" or "Increase in profits from selling crops; thousands of USD; 12", etc. If no Indicator is reported, return instead "Not reported; NA; NA".</t>
-    </r>
-  </si>
-  <si>
     <t>**Parameter:** Link or DOI.
 **Description:** Extract the DOI or URL that references to this article in its content.
 **Output Format:** Your response should be a string with the URL.</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
       <t>**</t>
     </r>
     <r>
@@ -671,7 +434,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** Primary Product Type.
+      <t>** Year of Report.
 **</t>
     </r>
     <r>
@@ -689,9 +452,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** The primary production of the agrifood system that the CGIAR center is studying. Identify the type of the primary product and then categorize it based on the vocabulary used in AGROVOC. For example:
-- (1) Cultivation of crops (e.g. cereals, legumes, fruits, and vegetables)
-- (2) Rearing of livestock (e.g. cattle, poultry, fish, other animal species) for food, feed, fiber, and bioenergy
+      <t>** The date on which the study/document was published. Don't get confused by the year the report was generated or accepted, it is the initial publishing date what you need to capture.
 **</t>
     </r>
     <r>
@@ -709,16 +470,11 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** Your response should be a string with the categorization for the primary product type, identifying the product and where applicable, its purpose. For example "Cultivation of crops (legumes)" or "Rearing of livesock (cattle) for food". Use your judgement and AGROVOC vocabulary for the response wording.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
+      <t>** Output a single 4 digit year. E.g. "2002"</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>**</t>
     </r>
     <r>
@@ -736,7 +492,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** Category for Natural Resource Management.
+      <t>** Country of Study.
 **</t>
     </r>
     <r>
@@ -754,37 +510,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** The study would identify the practices that the CGIAR center is studying. These practices regard in general the stewardship of ecosystems, biodiversity, soil health, water systems, and climate resilience to ensure sustainable food production. You have to go through the document/content and identify the main practices the study identified, is concerned about; or to which its content/impact is related. You should then assign one of the categories below and return that as your answer. Some categories are general, like "Crop management" while others are more specific, like "Crop management - agroforestry." Assign first the general category to the Natural Resource Management practices identified in the study and then do another pass to see if there is enough information to apply instead one of the more specific labels/categories. The categories are:
-- Aquaculture
-- Crop management
-- Crop management - agroecological practices
-- Crop management - agroforestry
-- Crop management - conservation agricultural practices
-- Crop management - crop roatations
-- Crop management - disease and pest management
-- Crop management - farmer knowledge
-- Crop management - gender roles and farm labour availability
-- Crop management - improved varieties
-- Crop management - smallholder farmers
-- Crop management - soil health
-- Crop management - technological adoption
-- Crop management - varietal adoption
-- Crop management - weather and climate services
-- Crop management technologies - improved practices
-- Farm management
-- Farm management - agroforestry
-- Farm management - climate advisories
-- Farm management - climate smart agriculture
-- Farm management - humanitarian support
-- Forestry management
-- Livestock management
-- Livestock management - animal health
-- Livestock management - fodder adoption
-- Livestock management - improved strains
-- Livestock management - livestock asset transfer
-- Post harvest - nutrition studies
-- Value chains
-- Value chains - agribusiness
+      <t>** The name of the country where the study/observations took place.
 **</t>
     </r>
     <r>
@@ -802,16 +528,11 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>** Return a single category from the ones above as your response.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
+      <t>** Reply with the name of the country, e.g. "Spain". If the study took place in more than one country, then list the different countries separated by commas, for example "Ghana, Ethiopia". Don't output names of regions or aggregations such as "10 African countries" just country names separated by commas.</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>**</t>
     </r>
     <r>
@@ -820,65 +541,120 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
-      </rPr>
-      <t>Parameter:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Study Theme.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Description:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** The main topic/theme of the study; which is the attribution/contribution of CGIAR interventions/policies/innovations by a CGIAR center. There are no predefined categories for this parameter.
-**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Output Format:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>** Your answer should be in the format of a short title that outlines the theme.</t>
-    </r>
-  </si>
-  <si>
-    <t>**Parameter:** Crops.
-**Description:** Create a list of any of the crops mentioned in the text.
-**Output Format:** Your response should be a string with values separated by commas.</t>
+        <family val="2"/>
+      </rPr>
+      <t>Parameter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>:** Contributing Initiatives or centers.
+**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Description</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">:** CGIAR is associated with multiple Initiatives and Centers. You need to extract the names of the ones mentioned in the text, if any.
+**Output Format:** Your response should be a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>string with values separated by commas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>. For example "CIMMYT, AgriLac Resiliente, ICARDA".
+Here is the list of values that you could find in the text that you should capture, this is the complete list of CGIAR initiaitves and centers:
+"[
+  { "name": "Africa Rice Center", "acronym": "AfricaRice" },
+  { "name": "Alliance of Bioversity and CIAT - Headquarter (Bioversity International)", "acronym": "ABC" },
+  { "name": "Alliance of Bioversity and CIAT - Regional Hub (Centro Internacional de Agricultura Tropical)", "acronym": "ABC" },
+  { "name": "Center for International Forestry Research", "acronym": "CIFOR" },
+  { "name": "Centro Internacional de Mejoramiento de Maíz y Trigo", "acronym": "CIMMYT" },
+  { "name": "Centro Internacional de la Papa", "acronym": "CIP" },
+  { "name": "International Center for Agricultural Research in the Dry Areas", "acronym": "ICARDA" },
+  { "name": "World Agroforestry Centre", "acronym": "ICRAF" },
+  { "name": "International Crops Research Institute for the Semi-Arid Tropics", "acronym": "ICRISAT" },
+  { "name": "International Food Policy Research institute", "acronym": "IFPRI" },
+  { "name": "International Institute of Tropical Agriculture", "acronym": "IITA" },
+  { "name": "International Livestock Research Institute", "acronym": "ILRI" },
+  { "name": "International Rice Research Institute", "acronym": "IRRI" },
+  { "name": "International Water Management Institute", "acronym": "IWMI" },
+  { "name": "WorldFish", "acronym": "WorldFish" },
+  { "name": "System Organization", "acronym": "SO" },
+  { "name": "Accelerated Breeding", "acronym": "Accelerated Breeding" },
+  { "name": "Genebanks", "acronym": "Genebanks" },
+  { "name": "Breeding Resources", "acronym": "Breeding Resources" },
+  { "name": "Market Intelligence", "acronym": "Market Intelligence" },
+  { "name": "Seed Equal", "acronym": "Seed Equal" },
+  { "name": "Protecting Human Health Through a One Health Approach", "acronym": "One Health" },
+  { "name": "ActioNs for Innovative climate change Mitigation &amp; Adaptation of Livestock Systems (ANIMALS)", "acronym": "ActioNs for Innovative climate change Mitigation &amp; Adaptation of Livestock Systems (ANIMALS)" },
+  { "name": "ASPIRE - building integrated agrisilvopastoral food systems resilient to climate change and other crises", "acronym": "ASPIRE - building integrated agrisilvopastoral food systems resilient to climate change and other crises" },
+  { "name": "From Fragility to Resilience in Central and West Asia and North Africa", "acronym": "Fragility to Resilience in Central and West Asia and North Africa" },
+  { "name": "Excellence in Agronomy for Sustainable Intensification and Climate Change Adaptation", "acronym": "Excellence in Agronomy" },
+  { "name": "Nature-Positive Solutions for Shifting Agrifood Systems to More Resilient and Sustainable Pathways", "acronym": "Nature-Positive Solutions" },
+  { "name": "Plant Health and Rapid Response to Protect Food Security and Livelihoods", "acronym": "Plant Health" },
+  { "name": "AgriLAC Resiliente: Resilient Agrifood Innovation Systems in Latin America and the Caribbean", "acronym": "AgriLAC Resiliente" },
+  { "name": "Resilient Aquatic Food Systems for Healthy People and Planet", "acronym": "Aquatic Foods" },
+  { "name": "Resilient Cities Through Sustainable Urban and Peri-Urban Agrifood Systems", "acronym": "Resilient Cities" },
+  { "name": "Sustainable Animal Productivity for Livelihoods, Nutrition and Gender Inclusion", "acronym": "Sustainable Animal Productivity" },
+  { "name": "Securing the Food Systems of Asian Mega-Deltas for Climate and Livelihood Resilience", "acronym": "Asian Mega-Deltas" },
+  { "name": "Sustainable Intensification of Mixed Farming Systems", "acronym": "Mixed Farming Systems" },
+  { "name": "Transforming Agrifood Systems in South Asia", "acronym": "Transforming Agrifood Systems in South Asia" },
+  { "name": "Ukama Ustawi: Diversification for Resilient Agrifood Systems in East and Southern Africa", "acronym": "Diversification in East and Southern Africa" },
+  { "name": "Transforming AgriFood Systems in West and Central Africa", "acronym": "West and Central African Food Systems Transformation" },
+  { "name": "ClimBeR: Building Systemic Resilience Against Climate Variability and Extremes", "acronym": "Climate Resilience" },
+  { "name": "Foresight and Metrics to Accelerate Food, Land, and Water Systems Transformation", "acronym": "Foresight" },
+  { "name": "Digital Innovation and Transformation", "acronym": "Digital Innovation" },
+  { "name": "Harnessing Gender and Social Equality for Resilience in Agrifood Systems", "acronym": "Gender Equality" },
+  { "name": "National Policies and Strategies for Food, Land and Water Systems Transformation", "acronym": "National Policies and Strategies" },
+  { "name": "NEXUS Gains: Realizing Multiple Benefits Across Water, Energy, Food and Ecosystems", "acronym": "NEXUS Gains" },
+  { "name": "Rethinking Food Markets and Value Chains for Inclusion and Sustainability", "acronym": "Rethinking Food Markets" },
+  { "name": "Sustainable Healthy Diets through Food Systems Transformation", "acronym": "Sustainable Healthy Diets" },
+  { "name": "Transformational Agroecology across Food, Land, and Water systems", "acronym": "Agroecology" },
+  { "name": "Mitigate+: Research for Low-Emission Food Systems", "acronym": "Low-Emission Food Systems" },
+  { "name": "Fruit and Vegetables for Sustainable Healthy Diets", "acronym": "Fruit and Vegetables for Sustainable Healthy Diets" },
+  { "name": "Livestock, Climate and System Resilience", "acronym": "Livestock and Climate" },
+  { "name": "Fragility, Conflict and Migration", "acronym": "Fragility, Conflict and Migration" },
+  { "name": "GENDER Impact Platform", "acronym": "GENDER Impact Platform" },
+  { "name": "Climate Adaptation and Mitigation Impact Area Platform", "acronym": "Climate Platform" },
+  { "name": "Environment and Biodiversity Impact Area Platform", "acronym": "Environment and Biodiversity Impact Area Platform" },
+  { "name": "NUTRITION Impact Platform", "acronym": "NUTRITION Impact Platform" },
+  { "name": "Accelerating Crop Improvement Through Genome Editing", "acronym": "Genome Editing" }
+]"</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -890,12 +666,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="&quot;Aptos Narrow&quot;"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
@@ -933,18 +703,12 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -971,7 +735,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -982,25 +746,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1222,91 +977,69 @@
     <tabColor rgb="FFF1C232"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.3984375" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="21.5703125" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" customWidth="1"/>
-    <col min="7" max="7" width="71.5703125" customWidth="1"/>
-    <col min="8" max="9" width="21.5703125" customWidth="1"/>
-    <col min="14" max="14" width="21.5703125" customWidth="1"/>
-    <col min="16" max="16" width="21.5703125" customWidth="1"/>
-    <col min="17" max="17" width="57.28515625" customWidth="1"/>
-    <col min="18" max="18" width="21.5703125" customWidth="1"/>
+    <col min="1" max="2" width="21.59765625" customWidth="1"/>
+    <col min="5" max="5" width="21.59765625" customWidth="1"/>
+    <col min="7" max="7" width="71.59765625" customWidth="1"/>
+    <col min="8" max="9" width="21.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" customHeight="1">
+    <row r="1" spans="1:14" ht="15.75" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="E1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
     </row>
-    <row r="2" spans="1:19" ht="338.25" customHeight="1">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:14" ht="338.25" customHeight="1">
+      <c r="A2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="H2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="J2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="K2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="L2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="M2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="N2" s="5" t="s">
         <v>10</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="P2" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>